<commit_message>
feat(F-NAR-019): TREE-AUT-020 polish Le chat à la fenêtre d'Amir
Alignement xlsx sur merged vocal (anneau de pollen).
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-020.xlsx
+++ b/stories/arbres/TREE-AUT-020.xlsx
@@ -1980,17 +1980,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Amir se baisse vers le coussin. Il le reprend, grain par grain. Je le reprends, il est à moi. Merci, Amir. Tu le portes, sans courir ? Oui, je reste. Un grain orange reste sur le tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le bac garde un creux, vide.</t>
+          <t>Amir se baisse vers le coussin rayé. Il le reprend, grain par grain. Je le reprends, il est à moi. Merci, Amir. Tu le portes, sans courir ? Oui, je reste. Un grain orange reste sur le tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le bac garde un creux, vide.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir se baisse vers le coussin. Il le reprend, grain par grain. Je le reprends, il est à moi. Merci, Amir. Tu le portes, sans courir ? Oui, je reste. Un grain orange reste sur le tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le bac garde un creux, vide.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir se baisse vers le &lt;emphasis level="moderate"&gt;coussin rayé&lt;/emphasis&gt;. Il le reprend, grain par grain. Je le reprends, il est à moi. Merci, Amir. Tu le portes, sans courir ? Oui, je reste. Un grain orange reste sur le tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le bac garde un creux, vide.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Amir se baisse vers le coussin. Il le reprend, grain par grain. Je le reprends, il est à moi. Merci, Amir. Tu le portes, sans courir ? Oui, je reste. Un grain orange reste sur le tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le bac garde un creux, vide. [pause]</t>
+          <t>Amir se baisse vers le &lt;emphasis&gt;coussin rayé&lt;/emphasis&gt;. Il le reprend, grain par grain. Je le reprends, il est à moi. Merci, Amir. Tu le portes, sans courir ? Oui, je reste. Un grain orange reste sur le tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le bac garde un creux, vide. [pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="AH6" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>coussin rayé</t>
         </is>
       </c>
       <c r="AI6" s="2" t="n">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Amir se baisse vers le coussin.
+          <t>narrateur|Amir se baisse vers le coussin rayé.
 narrateur|Il le reprend, grain par grain.
 enfant-m|Je le reprends, il est à moi.
 papa|Merci, Amir.
@@ -2951,17 +2951,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Le rebord chaud porte le chat, enfin. Le coussin rayé a un grain de sable. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau de pollen dort sur la manche.</t>
+          <t>Le rebord chaud porte le chat, enfin. Le coussin rayé a un grain de sable. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. L'anneau de pollen dort sur la manche.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le rebord chaud porte le chat, enfin. Le coussin rayé a un grain de sable. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt; dort sur la manche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le rebord chaud porte le chat, enfin. Le coussin rayé a un grain de sable. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau de pollen dort sur la manche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le rebord chaud porte le chat, enfin. Le coussin rayé a un grain de sable. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt; dort sur la manche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le rebord chaud porte le chat, enfin. Le coussin rayé a un grain de sable. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau de pollen dort sur la manche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -3107,7 +3107,7 @@
 narrateur|Le ballon dort, loin des pattes.
 papa|On rentre, le manteau avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|L'anneau de pollen dort sur la manche.</t>
         </is>
@@ -3335,17 +3335,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Voilà le chat, près des chaussures brunes. Le coussin rayé a un grain, et un lacet. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau de pollen dore le lacet, minuscule.</t>
+          <t>Voilà le chat, près des chaussures brunes. Le coussin rayé a un grain, et un lacet. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. L'anneau de pollen dore le lacet, minuscule.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Voilà le chat, près des chaussures brunes. Le coussin rayé a un grain, et un lacet. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt; dore le lacet, minuscule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Voilà le chat, près des chaussures brunes. Le coussin rayé a un grain, et un lacet. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau de pollen dore le lacet, minuscule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Voilà le chat, près des chaussures brunes. Le coussin rayé a un grain, et un lacet. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt; dore le lacet, minuscule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Voilà le chat, près des chaussures brunes. Le coussin rayé a un grain, et un lacet. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau de pollen dore le lacet, minuscule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3491,7 +3491,7 @@
 narrateur|Le ballon dort, loin des pattes.
 maman|On rentre, les chaussures avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|L'anneau de pollen dore le lacet, minuscule.</t>
         </is>
@@ -3719,17 +3719,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Contre le sac, le chat se fait petit. Le coussin rayé a un grain, près du rabat. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau de pollen brille sur la sangle.</t>
+          <t>Contre le sac, le chat se fait petit. Le coussin rayé a un grain, près du rabat. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. L'anneau de pollen brille sur la sangle.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Contre le sac, le chat se fait petit. Le coussin rayé a un grain, près du rabat. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt; brille sur la sangle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Contre le sac, le chat se fait petit. Le coussin rayé a un grain, près du rabat. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau de pollen brille sur la sangle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Contre le sac, le chat se fait petit. Le coussin rayé a un grain, près du rabat. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt; brille sur la sangle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Contre le sac, le chat se fait petit. Le coussin rayé a un grain, près du rabat. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau de pollen brille sur la sangle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -3875,7 +3875,7 @@
 narrateur|Le ballon dort, loin des pattes.
 papa|On rentre, le sac avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|L'anneau de pollen brille sur la sangle.</t>
         </is>
@@ -4496,17 +4496,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Au chaud, le chat a choisi le nid. Le coussin rayé sent le seau, et le col. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un cercle orange reste au col, secret.</t>
+          <t>Au chaud, le chat a choisi le nid. Le coussin rayé sent le seau, et le col. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Un cercle orange reste au col, secret.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au chaud, le chat a choisi le nid. Le coussin rayé sent le seau, et le col. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un cercle orange reste au col, secret.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au chaud, le chat a choisi le nid. Le coussin rayé sent le seau, et le col. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un cercle orange reste au col, secret.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au chaud, le chat a choisi le nid. Le coussin rayé sent le seau, et le col. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un cercle orange reste au col, secret.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au chaud, le chat a choisi le nid. Le coussin rayé sent le seau, et le col. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un cercle orange reste au col, secret.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4589,7 +4589,11 @@
       <c r="AG19" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH19" s="2" t="inlineStr"/>
+      <c r="AH19" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI19" s="2" t="n">
         <v>0</v>
       </c>
@@ -4648,7 +4652,7 @@
 narrateur|Le seau dort, loin des pattes.
 papa|On rentre, le manteau avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Un cercle orange reste au col, secret.</t>
         </is>
@@ -4876,17 +4880,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Près du seau, le chat ferme un œil. Le coussin rayé sent le seau, et le cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un cercle orange dort dans le cuir.</t>
+          <t>Près du seau, le chat ferme un œil. Le coussin rayé sent le seau, et le cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Un cercle orange dort dans le cuir.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Près du seau, le chat ferme un œil. Le coussin rayé sent le seau, et le cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un cercle orange dort dans le cuir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Près du seau, le chat ferme un œil. Le coussin rayé sent le seau, et le cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un cercle orange dort dans le cuir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Près du seau, le chat ferme un œil. Le coussin rayé sent le seau, et le cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un cercle orange dort dans le cuir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Près du seau, le chat ferme un œil. Le coussin rayé sent le seau, et le cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un cercle orange dort dans le cuir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4969,7 +4973,11 @@
       <c r="AG21" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH21" s="2" t="inlineStr"/>
+      <c r="AH21" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI21" s="2" t="n">
         <v>0</v>
       </c>
@@ -5028,7 +5036,7 @@
 narrateur|Le seau dort, loin des pattes.
 maman|On rentre, les chaussures avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Un cercle orange dort dans le cuir.</t>
         </is>
@@ -5256,17 +5264,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Sous le rabat, un museau gris paraît. Le coussin rayé sent le seau, et le sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un cercle orange veille sur le rabat.</t>
+          <t>Sous le rabat, un museau gris paraît. Le coussin rayé sent le seau, et le sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Un cercle orange veille sur le rabat.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sous le rabat, un museau gris paraît. Le coussin rayé sent le seau, et le sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un cercle orange veille sur le rabat.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sous le rabat, un museau gris paraît. Le coussin rayé sent le seau, et le sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un cercle orange veille sur le rabat.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sous le rabat, un museau gris paraît. Le coussin rayé sent le seau, et le sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un cercle orange veille sur le rabat.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sous le rabat, un museau gris paraît. Le coussin rayé sent le seau, et le sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un cercle orange veille sur le rabat.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5349,7 +5357,11 @@
       <c r="AG23" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH23" s="2" t="inlineStr"/>
+      <c r="AH23" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI23" s="2" t="n">
         <v>0</v>
       </c>
@@ -5408,7 +5420,7 @@
 narrateur|Le seau dort, loin des pattes.
 papa|On rentre, le sac avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Un cercle orange veille sur le rabat.</t>
         </is>
@@ -6029,17 +6041,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Le doudou veille, le chat est au nid. Le coussin rayé a l'oreille grise, collée. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre à la manche.</t>
+          <t>Le doudou veille, le chat est au nid. Le coussin rayé a l'oreille grise, collée. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre à la manche.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou veille, le chat est au nid. Le coussin rayé a l'oreille grise, collée. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre à la manche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou veille, le chat est au nid. Le coussin rayé a l'oreille grise, collée. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre à la manche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou veille, le chat est au nid. Le coussin rayé a l'oreille grise, collée. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre à la manche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou veille, le chat est au nid. Le coussin rayé a l'oreille grise, collée. Il est venu, presque pas. Le jardin des trois coins se tait. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre à la manche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6122,7 +6134,11 @@
       <c r="AG27" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH27" s="2" t="inlineStr"/>
+      <c r="AH27" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI27" s="2" t="n">
         <v>0</v>
       </c>
@@ -6181,7 +6197,7 @@
 narrateur|Le doudou dort, loin des pattes.
 papa|On rentre, le manteau avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Voilà le pollen, parti du verre à la manche.</t>
         </is>
@@ -6409,17 +6425,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>L'oreille grise pend, près des souliers. Le coussin rayé a l'oreille, près du cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au lacet.</t>
+          <t>L'oreille grise pend, près des souliers. Le coussin rayé a l'oreille, près du cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au lacet.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oreille grise pend, près des souliers. Le coussin rayé a l'oreille, près du cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au lacet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oreille grise pend, près des souliers. Le coussin rayé a l'oreille, près du cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au lacet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oreille grise pend, près des souliers. Le coussin rayé a l'oreille, près du cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au lacet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oreille grise pend, près des souliers. Le coussin rayé a l'oreille, près du cuir. J'ai attendu, et il est venu. Le jardin des trois coins se tait. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au lacet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6502,7 +6518,11 @@
       <c r="AG29" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH29" s="2" t="inlineStr"/>
+      <c r="AH29" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI29" s="2" t="n">
         <v>0</v>
       </c>
@@ -6561,7 +6581,7 @@
 narrateur|Le doudou dort, loin des pattes.
 maman|On rentre, les chaussures avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Voilà le pollen, parti du verre au lacet.</t>
         </is>
@@ -6789,17 +6809,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Dans le sac, le chat se tait. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au sac.</t>
+          <t>Dans le sac, le chat se tait. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au sac.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans le sac, le chat se tait. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Dans le sac, le chat se tait. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans le sac, le chat se tait. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Dans le sac, le chat se tait. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. Le jardin des trois coins se tait. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voilà le pollen, parti du verre au sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -6882,7 +6902,11 @@
       <c r="AG31" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH31" s="2" t="inlineStr"/>
+      <c r="AH31" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI31" s="2" t="n">
         <v>0</v>
       </c>
@@ -6941,7 +6965,7 @@
 narrateur|Le doudou dort, loin des pattes.
 papa|On rentre, le sac avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Voilà le pollen, parti du verre au sac.</t>
         </is>
@@ -7355,17 +7379,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Amir ramasse le coussin, au bas. Il le reprend, contre lui. Je le reprends, il est froid. Bravo, Amir. Tu le portes, sans glisser ? Oui, je marche. Une feuille reste collée au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le métal se tait, un instant.</t>
+          <t>Amir ramasse le coussin rayé, au bas. Il le reprend, contre lui. Je le reprends, il est froid. Bravo, Amir. Tu le portes, sans glisser ? Oui, je marche. Une feuille reste collée au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le métal se tait, un instant.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir ramasse le coussin, au bas. Il le reprend, contre lui. Je le reprends, il est froid. Bravo, Amir. Tu le portes, sans glisser ? Oui, je marche. Une feuille reste collée au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le métal se tait, un instant.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir ramasse le &lt;emphasis level="moderate"&gt;coussin rayé&lt;/emphasis&gt;, au bas. Il le reprend, contre lui. Je le reprends, il est froid. Bravo, Amir. Tu le portes, sans glisser ? Oui, je marche. Une feuille reste collée au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le métal se tait, un instant.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Amir ramasse le coussin, au bas. Il le reprend, contre lui. Je le reprends, il est froid. Bravo, Amir. Tu le portes, sans glisser ? Oui, je marche. Une feuille reste collée au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le métal se tait, un instant. [pause]</t>
+          <t>Amir ramasse le &lt;emphasis&gt;coussin rayé&lt;/emphasis&gt;, au bas. Il le reprend, contre lui. Je le reprends, il est froid. Bravo, Amir. Tu le portes, sans glisser ? Oui, je marche. Une feuille reste collée au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. Le métal se tait, un instant. [pause]</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7446,7 +7470,7 @@
       </c>
       <c r="AH34" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>coussin rayé</t>
         </is>
       </c>
       <c r="AI34" s="2" t="n">
@@ -7499,7 +7523,7 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>narrateur|Amir ramasse le coussin, au bas.
+          <t>narrateur|Amir ramasse le coussin rayé, au bas.
 narrateur|Il le reprend, contre lui.
 enfant-m|Je le reprends, il est froid.
 maman|Bravo, Amir.
@@ -8326,17 +8350,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Après le métal, le rebord est doux. Le coussin rayé a une feuille de rampe. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au tissu.</t>
+          <t>Après le métal, le rebord est doux. Le coussin rayé a une feuille de rampe. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au tissu.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Après le métal, le rebord est doux. Le coussin rayé a une feuille de rampe. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au tissu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Après le métal, le rebord est doux. Le coussin rayé a une feuille de rampe. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au tissu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Après le métal, le rebord est doux. Le coussin rayé a une feuille de rampe. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au tissu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Après le métal, le rebord est doux. Le coussin rayé a une feuille de rampe. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au tissu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8419,7 +8443,11 @@
       <c r="AG39" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH39" s="2" t="inlineStr"/>
+      <c r="AH39" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI39" s="2" t="n">
         <v>0</v>
       </c>
@@ -8478,7 +8506,7 @@
 narrateur|Le ballon dort, loin des pattes.
 papa|On rentre, le manteau avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|L'anneau orange a glissé du métal au tissu.</t>
         </is>
@@ -8706,17 +8734,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Au bas des marches, le chat s'installe. Le coussin rayé a une feuille, et le lacet. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au lacet.</t>
+          <t>Au bas des marches, le chat s'installe. Le coussin rayé a une feuille, et le lacet. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au lacet.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au bas des marches, le chat s'installe. Le coussin rayé a une feuille, et le lacet. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au lacet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au bas des marches, le chat s'installe. Le coussin rayé a une feuille, et le lacet. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au lacet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au bas des marches, le chat s'installe. Le coussin rayé a une feuille, et le lacet. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au lacet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au bas des marches, le chat s'installe. Le coussin rayé a une feuille, et le lacet. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au lacet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8799,7 +8827,11 @@
       <c r="AG41" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH41" s="2" t="inlineStr"/>
+      <c r="AH41" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI41" s="2" t="n">
         <v>0</v>
       </c>
@@ -8858,7 +8890,7 @@
 narrateur|Le ballon dort, loin des pattes.
 maman|On rentre, les chaussures avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|L'anneau orange a glissé du métal au lacet.</t>
         </is>
@@ -9086,17 +9118,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Le sac beige tient un secret gris. Le coussin rayé a une feuille, près du sac. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au sac.</t>
+          <t>Le sac beige tient un secret gris. Le coussin rayé a une feuille, près du sac. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au sac.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le sac beige tient un secret gris. Le coussin rayé a une feuille, près du sac. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le sac beige tient un secret gris. Le coussin rayé a une feuille, près du sac. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le sac beige tient un secret gris. Le coussin rayé a une feuille, près du sac. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le sac beige tient un secret gris. Le coussin rayé a une feuille, près du sac. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. L'anneau orange a glissé du métal au sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9179,7 +9211,11 @@
       <c r="AG43" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH43" s="2" t="inlineStr"/>
+      <c r="AH43" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI43" s="2" t="n">
         <v>0</v>
       </c>
@@ -9238,7 +9274,7 @@
 narrateur|Le ballon dort, loin des pattes.
 papa|On rentre, le sac avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|L'anneau orange a glissé du métal au sac.</t>
         </is>
@@ -9859,17 +9895,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Le seau sonne, loin du nid bleu. Le coussin rayé a une goutte, au col. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au col, fine.</t>
+          <t>Le seau sonne, loin du nid bleu. Le coussin rayé a une goutte, au col. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au col, fine.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau sonne, loin du nid bleu. Le coussin rayé a une goutte, au col. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au col, fine.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau sonne, loin du nid bleu. Le coussin rayé a une goutte, au col. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au col, fine.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau sonne, loin du nid bleu. Le coussin rayé a une goutte, au col. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au col, fine.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau sonne, loin du nid bleu. Le coussin rayé a une goutte, au col. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au col, fine.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9952,7 +9988,11 @@
       <c r="AG47" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH47" s="2" t="inlineStr"/>
+      <c r="AH47" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI47" s="2" t="n">
         <v>0</v>
       </c>
@@ -10011,7 +10051,7 @@
 narrateur|Le seau dort, loin des pattes.
 papa|On rentre, le manteau avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Une poussière orange sèche au col, fine.</t>
         </is>
@@ -10239,17 +10279,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Une goutte sèche, près du cuir brun. Le coussin rayé a une goutte, au cuir. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au cuir, fine.</t>
+          <t>Une goutte sèche, près du cuir brun. Le coussin rayé a une goutte, au cuir. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au cuir, fine.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une goutte sèche, près du cuir brun. Le coussin rayé a une goutte, au cuir. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au cuir, fine.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une goutte sèche, près du cuir brun. Le coussin rayé a une goutte, au cuir. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au cuir, fine.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une goutte sèche, près du cuir brun. Le coussin rayé a une goutte, au cuir. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au cuir, fine.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une goutte sèche, près du cuir brun. Le coussin rayé a une goutte, au cuir. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au cuir, fine.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10332,7 +10372,11 @@
       <c r="AG49" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH49" s="2" t="inlineStr"/>
+      <c r="AH49" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI49" s="2" t="n">
         <v>0</v>
       </c>
@@ -10391,7 +10435,7 @@
 narrateur|Le seau dort, loin des pattes.
 maman|On rentre, les chaussures avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Une poussière orange sèche au cuir, fine.</t>
         </is>
@@ -10619,17 +10663,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Le seau cale le sac, le chat dedans. Le coussin rayé a une goutte, au rabat. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au rabat, fine.</t>
+          <t>Le seau cale le sac, le chat dedans. Le coussin rayé a une goutte, au rabat. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au rabat, fine.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau cale le sac, le chat dedans. Le coussin rayé a une goutte, au rabat. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au rabat, fine.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau cale le sac, le chat dedans. Le coussin rayé a une goutte, au rabat. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au rabat, fine.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau cale le sac, le chat dedans. Le coussin rayé a une goutte, au rabat. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au rabat, fine.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau cale le sac, le chat dedans. Le coussin rayé a une goutte, au rabat. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Une poussière orange sèche au rabat, fine.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10712,7 +10756,11 @@
       <c r="AG51" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH51" s="2" t="inlineStr"/>
+      <c r="AH51" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI51" s="2" t="n">
         <v>0</v>
       </c>
@@ -10771,7 +10819,7 @@
 narrateur|Le seau dort, loin des pattes.
 papa|On rentre, le sac avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Une poussière orange sèche au rabat, fine.</t>
         </is>
@@ -11392,17 +11440,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a vu le manteau, puis le chat. Le coussin rayé a le doudou, et le bleu. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voici le verre nu, le manteau garde l'anneau.</t>
+          <t>Le doudou a vu le manteau, puis le chat. Le coussin rayé a le doudou, et le bleu. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Voici le verre nu, le manteau garde l'anneau.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou a vu le manteau, puis le chat. Le coussin rayé a le doudou, et le bleu. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voici le verre nu, le manteau garde l'anneau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou a vu le manteau, puis le chat. Le coussin rayé a le doudou, et le bleu. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voici le verre nu, le manteau garde l'anneau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou a vu le manteau, puis le chat. Le coussin rayé a le doudou, et le bleu. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voici le verre nu, le manteau garde l'anneau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou a vu le manteau, puis le chat. Le coussin rayé a le doudou, et le bleu. Il est venu, presque pas. Le métal se tait, lui aussi. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voici le verre nu, le manteau garde l'anneau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11485,7 +11533,11 @@
       <c r="AG55" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH55" s="2" t="inlineStr"/>
+      <c r="AH55" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI55" s="2" t="n">
         <v>0</v>
       </c>
@@ -11544,7 +11596,7 @@
 narrateur|Le doudou dort, loin des pattes.
 papa|On rentre, le manteau avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Voici le verre nu, le manteau garde l'anneau.</t>
         </is>
@@ -11772,17 +11824,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>L'oreille molle touche un lacet, puis se tait. Le coussin rayé a le doudou, et le brun. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voici le verre nu, le lacet garde l'anneau.</t>
+          <t>L'oreille molle touche un lacet, puis se tait. Le coussin rayé a le doudou, et le brun. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Voici le verre nu, le lacet garde l'anneau.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oreille molle touche un lacet, puis se tait. Le coussin rayé a le doudou, et le brun. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voici le verre nu, le lacet garde l'anneau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oreille molle touche un lacet, puis se tait. Le coussin rayé a le doudou, et le brun. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voici le verre nu, le lacet garde l'anneau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oreille molle touche un lacet, puis se tait. Le coussin rayé a le doudou, et le brun. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voici le verre nu, le lacet garde l'anneau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oreille molle touche un lacet, puis se tait. Le coussin rayé a le doudou, et le brun. J'ai attendu, et il est venu. Le métal se tait, lui aussi. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voici le verre nu, le lacet garde l'anneau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11865,7 +11917,11 @@
       <c r="AG57" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH57" s="2" t="inlineStr"/>
+      <c r="AH57" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI57" s="2" t="n">
         <v>0</v>
       </c>
@@ -11924,7 +11980,7 @@
 narrateur|Le doudou dort, loin des pattes.
 maman|On rentre, les chaussures avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Voici le verre nu, le lacet garde l'anneau.</t>
         </is>
@@ -12152,17 +12208,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Près du métal, le sac garde le chat. Le coussin rayé a le doudou, et le beige. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voici le verre nu, le sac garde l'anneau.</t>
+          <t>Près du métal, le sac garde le chat. Le coussin rayé a le doudou, et le beige. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Voici le verre nu, le sac garde l'anneau.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Près du métal, le sac garde le chat. Le coussin rayé a le doudou, et le beige. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voici le verre nu, le sac garde l'anneau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Près du métal, le sac garde le chat. Le coussin rayé a le doudou, et le beige. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voici le verre nu, le sac garde l'anneau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Près du métal, le sac garde le chat. Le coussin rayé a le doudou, et le beige. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Voici le verre nu, le sac garde l'anneau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Près du métal, le sac garde le chat. Le coussin rayé a le doudou, et le beige. Le tic s'est tu, papa. Le métal se tait, lui aussi. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Voici le verre nu, le sac garde l'anneau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12245,7 +12301,11 @@
       <c r="AG59" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH59" s="2" t="inlineStr"/>
+      <c r="AH59" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI59" s="2" t="n">
         <v>0</v>
       </c>
@@ -12304,7 +12364,7 @@
 narrateur|Le doudou dort, loin des pattes.
 papa|On rentre, le sac avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Voici le verre nu, le sac garde l'anneau.</t>
         </is>
@@ -12718,17 +12778,17 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Amir reprend le coussin, sur le bois. Il le secoue, sans pousser le siège. Je le reprends, il est à moi. Oui, tes mains sont prêtes. Tu le portes, sans balancer ? Oui, je reste. Un brin de corde reste au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. La corde retombe, sans bruit.</t>
+          <t>Amir reprend le coussin rayé, sur le bois. Il le secoue, sans pousser le siège. Je le reprends, il est à moi. Oui, tes mains sont prêtes. Tu le portes, sans balancer ? Oui, je reste. Un brin de corde reste au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. La corde retombe, sans bruit.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir reprend le coussin, sur le bois. Il le secoue, sans pousser le siège. Je le reprends, il est à moi. Oui, tes mains sont prêtes. Tu le portes, sans balancer ? Oui, je reste. Un brin de corde reste au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. La corde retombe, sans bruit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir reprend le &lt;emphasis level="moderate"&gt;coussin rayé&lt;/emphasis&gt;, sur le bois. Il le secoue, sans pousser le siège. Je le reprends, il est à moi. Oui, tes mains sont prêtes. Tu le portes, sans balancer ? Oui, je reste. Un brin de corde reste au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. La corde retombe, sans bruit.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Amir reprend le coussin, sur le bois. Il le secoue, sans pousser le siège. Je le reprends, il est à moi. Oui, tes mains sont prêtes. Tu le portes, sans balancer ? Oui, je reste. Un brin de corde reste au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. La corde retombe, sans bruit. [pause]</t>
+          <t>Amir reprend le &lt;emphasis&gt;coussin rayé&lt;/emphasis&gt;, sur le bois. Il le secoue, sans pousser le siège. Je le reprends, il est à moi. Oui, tes mains sont prêtes. Tu le portes, sans balancer ? Oui, je reste. Un brin de corde reste au tissu. Le chat observe, loin, dans l'herbe. J'attends, moi aussi. La corde retombe, sans bruit. [pause]</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -12809,7 +12869,7 @@
       </c>
       <c r="AH62" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>coussin rayé</t>
         </is>
       </c>
       <c r="AI62" s="2" t="n">
@@ -12862,7 +12922,7 @@
       </c>
       <c r="AW62" t="inlineStr">
         <is>
-          <t>narrateur|Amir reprend le coussin, sur le bois.
+          <t>narrateur|Amir reprend le coussin rayé, sur le bois.
 narrateur|Il le secoue, sans pousser le siège.
 enfant-m|Je le reprends, il est à moi.
 papa|Oui, tes mains sont prêtes.
@@ -13689,17 +13749,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>La corde se tait, le chat est rentré. Le coussin rayé a un brin de corde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le bleu.</t>
+          <t>La corde se tait, le chat est rentré. Le coussin rayé a un brin de corde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le bleu.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La corde se tait, le chat est rentré. Le coussin rayé a un brin de corde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le bleu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La corde se tait, le chat est rentré. Le coussin rayé a un brin de corde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le bleu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La corde se tait, le chat est rentré. Le coussin rayé a un brin de corde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le bleu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La corde se tait, le chat est rentré. Le coussin rayé a un brin de corde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le ballon dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le bleu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13782,7 +13842,11 @@
       <c r="AG67" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH67" s="2" t="inlineStr"/>
+      <c r="AH67" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI67" s="2" t="n">
         <v>0</v>
       </c>
@@ -13841,7 +13905,7 @@
 narrateur|Le ballon dort, loin des pattes.
 papa|On rentre, le manteau avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Un tic lointain, puis l'anneau sur le bleu.</t>
         </is>
@@ -14069,17 +14133,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Un cling lointain, et les chaussures, et lui. Le coussin rayé a un brin, près du lacet. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le lacet.</t>
+          <t>Un cling lointain, et les chaussures, et lui. Le coussin rayé a un brin, près du lacet. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le lacet.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un cling lointain, et les chaussures, et lui. Le coussin rayé a un brin, près du lacet. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le lacet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un cling lointain, et les chaussures, et lui. Le coussin rayé a un brin, près du lacet. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le lacet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un cling lointain, et les chaussures, et lui. Le coussin rayé a un brin, près du lacet. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le lacet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un cling lointain, et les chaussures, et lui. Le coussin rayé a un brin, près du lacet. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le ballon dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le lacet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -14162,7 +14226,11 @@
       <c r="AG69" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH69" s="2" t="inlineStr"/>
+      <c r="AH69" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI69" s="2" t="n">
         <v>0</v>
       </c>
@@ -14221,7 +14289,7 @@
 narrateur|Le ballon dort, loin des pattes.
 maman|On rentre, les chaussures avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Un tic lointain, puis l'anneau sur le lacet.</t>
         </is>
@@ -14449,17 +14517,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Le sac beige a cessé de balancer. Le coussin rayé a un brin, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le beige.</t>
+          <t>Le sac beige a cessé de balancer. Le coussin rayé a un brin, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le beige.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le sac beige a cessé de balancer. Le coussin rayé a un brin, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le beige.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le sac beige a cessé de balancer. Le coussin rayé a un brin, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le beige.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le sac beige a cessé de balancer. Le coussin rayé a un brin, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le beige.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le sac beige a cessé de balancer. Le coussin rayé a un brin, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le ballon dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Un tic lointain, puis l'anneau sur le beige.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -14542,7 +14610,11 @@
       <c r="AG71" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH71" s="2" t="inlineStr"/>
+      <c r="AH71" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI71" s="2" t="n">
         <v>0</v>
       </c>
@@ -14601,7 +14673,7 @@
 narrateur|Le ballon dort, loin des pattes.
 papa|On rentre, le sac avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Un tic lointain, puis l'anneau sur le beige.</t>
         </is>
@@ -15222,17 +15294,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>L'anse froide a laissé le nid tranquille. Le coussin rayé a l'ombre du seau, ronde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au col.</t>
+          <t>L'anse froide a laissé le nid tranquille. Le coussin rayé a l'ombre du seau, ronde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au col.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'anse froide a laissé le nid tranquille. Le coussin rayé a l'ombre du seau, ronde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au col.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'anse froide a laissé le nid tranquille. Le coussin rayé a l'ombre du seau, ronde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au col.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'anse froide a laissé le nid tranquille. Le coussin rayé a l'ombre du seau, ronde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au col.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'anse froide a laissé le nid tranquille. Le coussin rayé a l'ombre du seau, ronde. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le seau dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au col.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15315,7 +15387,11 @@
       <c r="AG75" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH75" s="2" t="inlineStr"/>
+      <c r="AH75" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI75" s="2" t="n">
         <v>0</v>
       </c>
@@ -15374,7 +15450,7 @@
 narrateur|Le seau dort, loin des pattes.
 papa|On rentre, le manteau avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|La corde se tait, l'anneau reste au col.</t>
         </is>
@@ -15602,17 +15678,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Le seau pose son ombre, loin des pattes. Le coussin rayé a l'ombre du seau, au cuir. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au cuir.</t>
+          <t>Le seau pose son ombre, loin des pattes. Le coussin rayé a l'ombre du seau, au cuir. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au cuir.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau pose son ombre, loin des pattes. Le coussin rayé a l'ombre du seau, au cuir. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au cuir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le seau pose son ombre, loin des pattes. Le coussin rayé a l'ombre du seau, au cuir. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au cuir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau pose son ombre, loin des pattes. Le coussin rayé a l'ombre du seau, au cuir. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au cuir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le seau pose son ombre, loin des pattes. Le coussin rayé a l'ombre du seau, au cuir. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le seau dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au cuir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15695,7 +15771,11 @@
       <c r="AG77" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH77" s="2" t="inlineStr"/>
+      <c r="AH77" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI77" s="2" t="n">
         <v>0</v>
       </c>
@@ -15754,7 +15834,7 @@
 narrateur|Le seau dort, loin des pattes.
 maman|On rentre, les chaussures avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|La corde se tait, l'anneau reste au cuir.</t>
         </is>
@@ -15982,17 +16062,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Au pied de bois, le sac tient le chat. Le coussin rayé a l'ombre du seau, au rabat. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au rabat.</t>
+          <t>Au pied de bois, le sac tient le chat. Le coussin rayé a l'ombre du seau, au rabat. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au rabat.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au pied de bois, le sac tient le chat. Le coussin rayé a l'ombre du seau, au rabat. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au rabat.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Au pied de bois, le sac tient le chat. Le coussin rayé a l'ombre du seau, au rabat. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au rabat.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au pied de bois, le sac tient le chat. Le coussin rayé a l'ombre du seau, au rabat. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au rabat.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Au pied de bois, le sac tient le chat. Le coussin rayé a l'ombre du seau, au rabat. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le seau dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. La corde se tait, l'anneau reste au rabat.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -16075,7 +16155,11 @@
       <c r="AG79" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH79" s="2" t="inlineStr"/>
+      <c r="AH79" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI79" s="2" t="n">
         <v>0</v>
       </c>
@@ -16134,7 +16218,7 @@
 narrateur|Le seau dort, loin des pattes.
 papa|On rentre, le sac avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|La corde se tait, l'anneau reste au rabat.</t>
         </is>
@@ -16755,17 +16839,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>L'oreille grise veille, près du col bleu. Le coussin rayé a l'oreille, près du nid. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Sur le nid, l'anneau reste, tout net.</t>
+          <t>L'oreille grise veille, près du col bleu. Le coussin rayé a l'oreille, près du nid. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Sur le nid, l'anneau reste, tout net.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oreille grise veille, près du col bleu. Le coussin rayé a l'oreille, près du nid. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Sur le nid, l'anneau reste, tout net.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'oreille grise veille, près du col bleu. Le coussin rayé a l'oreille, près du nid. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Sur le nid, l'anneau reste, tout net.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oreille grise veille, près du col bleu. Le coussin rayé a l'oreille, près du nid. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Sur le nid, l'anneau reste, tout net.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'oreille grise veille, près du col bleu. Le coussin rayé a l'oreille, près du nid. Il est venu, presque pas. La corde se tait, maintenant. Le manteau bleu fait nid, sous lui. Le doudou dort, loin des pattes. On rentre, le manteau avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Sur le nid, l'anneau reste, tout net.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16848,7 +16932,11 @@
       <c r="AG83" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH83" s="2" t="inlineStr"/>
+      <c r="AH83" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI83" s="2" t="n">
         <v>0</v>
       </c>
@@ -16907,7 +16995,7 @@
 narrateur|Le doudou dort, loin des pattes.
 papa|On rentre, le manteau avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Sur le nid, l'anneau reste, tout net.</t>
         </is>
@@ -17135,17 +17223,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Le doudou chauffe, les chaussures aussi. Le coussin rayé a l'oreille, près des souliers. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Près des souliers, l'anneau reste, tout net.</t>
+          <t>Le doudou chauffe, les chaussures aussi. Le coussin rayé a l'oreille, près des souliers. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Près des souliers, l'anneau reste, tout net.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou chauffe, les chaussures aussi. Le coussin rayé a l'oreille, près des souliers. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Près des souliers, l'anneau reste, tout net.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le doudou chauffe, les chaussures aussi. Le coussin rayé a l'oreille, près des souliers. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Près des souliers, l'anneau reste, tout net.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou chauffe, les chaussures aussi. Le coussin rayé a l'oreille, près des souliers. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Près des souliers, l'anneau reste, tout net.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le doudou chauffe, les chaussures aussi. Le coussin rayé a l'oreille, près des souliers. J'ai attendu, et il est venu. La corde se tait, maintenant. Les chaussures brunes veillent, près de lui. Le doudou dort, loin des pattes. On rentre, les chaussures avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Près des souliers, l'anneau reste, tout net.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -17228,7 +17316,11 @@
       <c r="AG85" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH85" s="2" t="inlineStr"/>
+      <c r="AH85" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI85" s="2" t="n">
         <v>0</v>
       </c>
@@ -17287,7 +17379,7 @@
 narrateur|Le doudou dort, loin des pattes.
 maman|On rentre, les chaussures avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Près des souliers, l'anneau reste, tout net.</t>
         </is>
@@ -17515,17 +17607,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Trois tissus, et le chat au milieu. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Près du sac, l'anneau reste, tout net.</t>
+          <t>Trois tissus, et le chat au milieu. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'anneau de pollen. Sa poitrine se desserre, fière, calme. Près du sac, l'anneau reste, tout net.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Trois tissus, et le chat au milieu. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Près du sac, l'anneau reste, tout net.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Trois tissus, et le chat au milieu. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis level="moderate"&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Près du sac, l'anneau reste, tout net.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Trois tissus, et le chat au milieu. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin des pattes. Sa poitrine se desserre, fière, calme. Près du sac, l'anneau reste, tout net.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Trois tissus, et le chat au milieu. Le coussin rayé a l'oreille, près du sac. Le tic s'est tu, papa. La corde se tait, maintenant. Le sac beige fait grotte, autour de lui. Le doudou dort, loin des pattes. On rentre, le sac avec nous. Le chat aussi, sur le rebord. Amir pose une main, loin de l'&lt;emphasis&gt;anneau de pollen&lt;/emphasis&gt;. Sa poitrine se desserre, fière, calme. Près du sac, l'anneau reste, tout net.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17608,7 +17700,11 @@
       <c r="AG87" s="2" t="n">
         <v>-3</v>
       </c>
-      <c r="AH87" s="2" t="inlineStr"/>
+      <c r="AH87" s="2" t="inlineStr">
+        <is>
+          <t>anneau de pollen</t>
+        </is>
+      </c>
       <c r="AI87" s="2" t="n">
         <v>0</v>
       </c>
@@ -17667,7 +17763,7 @@
 narrateur|Le doudou dort, loin des pattes.
 papa|On rentre, le sac avec nous.
 enfant-m|Le chat aussi, sur le rebord.
-narrateur|Amir pose une main, loin des pattes.
+narrateur|Amir pose une main, loin de l'anneau de pollen.
 narrateur|Sa poitrine se desserre, fière, calme.
 narrateur|Près du sac, l'anneau reste, tout net.</t>
         </is>
@@ -17695,7 +17791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17808,6 +17904,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>